<commit_message>
v2 : update data progress
</commit_message>
<xml_diff>
--- a/data/UAT Scenarios - PRJ20260012 - Leadsync dan CRM.xlsx
+++ b/data/UAT Scenarios - PRJ20260012 - Leadsync dan CRM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03_QA_UAT_Dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{088921B1-AB1D-4B84-9EA3-4C1BDF662E1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FA76775-9DFA-495A-9EAA-DF3C3B055064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11224,11 +11224,11 @@
         <v>3</v>
       </c>
       <c r="D2" s="106">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E2" s="106" t="str">
         <f>IF(D2=0,"Open",IF(D2=C2,"Done","InProgress"))</f>
-        <v>Done</v>
+        <v>Open</v>
       </c>
       <c r="F2" s="106" t="str">
         <f>'UAT Scenarios'!H7</f>
@@ -11275,11 +11275,11 @@
         <v>3</v>
       </c>
       <c r="D3" s="106">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E3" s="106" t="str">
         <f t="shared" ref="E3:E26" si="0">IF(D3=0,"Open",IF(D3=C3,"Done","InProgress"))</f>
-        <v>Done</v>
+        <v>Open</v>
       </c>
       <c r="F3" s="106" t="str">
         <f>'UAT Scenarios'!H8</f>
@@ -11323,11 +11323,11 @@
         <v>3</v>
       </c>
       <c r="D4" s="106">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E4" s="106" t="str">
         <f t="shared" si="0"/>
-        <v>Done</v>
+        <v>Open</v>
       </c>
       <c r="F4" s="106" t="str">
         <f>'UAT Scenarios'!H9</f>
@@ -11375,11 +11375,11 @@
         <v>3</v>
       </c>
       <c r="D5" s="106">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E5" s="106" t="str">
         <f t="shared" si="0"/>
-        <v>Done</v>
+        <v>Open</v>
       </c>
       <c r="F5" s="106" t="str">
         <f>'UAT Scenarios'!H10</f>
@@ -11430,11 +11430,11 @@
         <v>2</v>
       </c>
       <c r="D6" s="106">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6" s="106" t="str">
         <f t="shared" si="0"/>
-        <v>Done</v>
+        <v>Open</v>
       </c>
       <c r="F6" s="106" t="str">
         <f>'UAT Scenarios'!H11</f>

</xml_diff>

<commit_message>
v3 : update all task done
</commit_message>
<xml_diff>
--- a/data/UAT Scenarios - PRJ20260012 - Leadsync dan CRM.xlsx
+++ b/data/UAT Scenarios - PRJ20260012 - Leadsync dan CRM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03_QA_UAT_Dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FA76775-9DFA-495A-9EAA-DF3C3B055064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69385F6C-D39A-49CE-9769-09A4AD468DAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3686,21 +3686,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="20" fillId="16" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3721,6 +3706,21 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="15" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -5082,6 +5082,104 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CF4DE456-0382-4233-97D9-C8D87CCD252D}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="J2:L7" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="7">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="5"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="Sum of Total Task" fld="2" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Task Done" fld="3" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="24">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="23">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="22">
+      <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="21">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="5" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="20">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="19">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="2">
+            <x v="0"/>
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A26540C3-E606-4EFB-8BF8-EE21F877AF12}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="P2:R8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="7">
@@ -5143,113 +5241,6 @@
     <dataField name="Count of Status" fld="4" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="10">
-    <format dxfId="28">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="27">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="26">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="25">
-      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="24">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="23">
-      <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="22">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="5" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="21">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="20">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="19">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CF4DE456-0382-4233-97D9-C8D87CCD252D}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="J2:L7" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="7">
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
-    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="5"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="2">
-    <dataField name="Sum of Total Task" fld="2" baseField="0" baseItem="0"/>
-    <dataField name="Sum of Task Done" fld="3" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="6">
     <format dxfId="34">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
@@ -5257,27 +5248,36 @@
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
     <format dxfId="32">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="31">
+      <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="30">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="29">
       <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="28">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="5" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="30">
+    <format dxfId="27">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="29">
+    <format dxfId="26">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
-          <reference field="4294967294" count="2">
-            <x v="0"/>
-            <x v="1"/>
-          </reference>
+          <reference field="4" count="0"/>
         </references>
       </pivotArea>
+    </format>
+    <format dxfId="25">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
@@ -8859,26 +8859,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="30.75" customHeight="1">
-      <c r="B1" s="166" t="s">
+      <c r="B1" s="172" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="166"/>
-      <c r="D1" s="166"/>
-      <c r="E1" s="166"/>
-      <c r="F1" s="166"/>
-      <c r="G1" s="166"/>
-      <c r="H1" s="166"/>
-      <c r="I1" s="166"/>
-      <c r="J1" s="166"/>
-      <c r="K1" s="166"/>
-      <c r="L1" s="166"/>
-      <c r="M1" s="166"/>
-      <c r="N1" s="166"/>
-      <c r="O1" s="166"/>
-      <c r="P1" s="166"/>
-      <c r="Q1" s="166"/>
-      <c r="R1" s="166"/>
-      <c r="S1" s="166"/>
+      <c r="C1" s="172"/>
+      <c r="D1" s="172"/>
+      <c r="E1" s="172"/>
+      <c r="F1" s="172"/>
+      <c r="G1" s="172"/>
+      <c r="H1" s="172"/>
+      <c r="I1" s="172"/>
+      <c r="J1" s="172"/>
+      <c r="K1" s="172"/>
+      <c r="L1" s="172"/>
+      <c r="M1" s="172"/>
+      <c r="N1" s="172"/>
+      <c r="O1" s="172"/>
+      <c r="P1" s="172"/>
+      <c r="Q1" s="172"/>
+      <c r="R1" s="172"/>
+      <c r="S1" s="172"/>
     </row>
     <row r="2" spans="1:19" s="125" customFormat="1" ht="27.75" customHeight="1">
       <c r="B2" s="123">
@@ -9020,18 +9020,18 @@
   <sheetData>
     <row r="1" spans="1:18">
       <c r="A1" s="88"/>
-      <c r="B1" s="165" t="s">
+      <c r="B1" s="173" t="s">
         <v>62</v>
       </c>
-      <c r="C1" s="165"/>
-      <c r="D1" s="165"/>
-      <c r="E1" s="165"/>
-      <c r="F1" s="165"/>
-      <c r="G1" s="165"/>
-      <c r="H1" s="165"/>
-      <c r="I1" s="165"/>
-      <c r="J1" s="165"/>
-      <c r="K1" s="165"/>
+      <c r="C1" s="173"/>
+      <c r="D1" s="173"/>
+      <c r="E1" s="173"/>
+      <c r="F1" s="173"/>
+      <c r="G1" s="173"/>
+      <c r="H1" s="173"/>
+      <c r="I1" s="173"/>
+      <c r="J1" s="173"/>
+      <c r="K1" s="173"/>
       <c r="L1" s="1"/>
       <c r="M1" s="89"/>
       <c r="N1" s="88"/>
@@ -9039,16 +9039,16 @@
     </row>
     <row r="2" spans="1:18" ht="42" customHeight="1">
       <c r="A2" s="88"/>
-      <c r="B2" s="165"/>
-      <c r="C2" s="165"/>
-      <c r="D2" s="165"/>
-      <c r="E2" s="165"/>
-      <c r="F2" s="165"/>
-      <c r="G2" s="165"/>
-      <c r="H2" s="165"/>
-      <c r="I2" s="165"/>
-      <c r="J2" s="165"/>
-      <c r="K2" s="165"/>
+      <c r="B2" s="173"/>
+      <c r="C2" s="173"/>
+      <c r="D2" s="173"/>
+      <c r="E2" s="173"/>
+      <c r="F2" s="173"/>
+      <c r="G2" s="173"/>
+      <c r="H2" s="173"/>
+      <c r="I2" s="173"/>
+      <c r="J2" s="173"/>
+      <c r="K2" s="173"/>
       <c r="L2" s="1"/>
       <c r="M2" s="89"/>
       <c r="N2" s="88"/>
@@ -9609,32 +9609,32 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:17" ht="14.4">
-      <c r="A3" s="167" t="s">
+      <c r="A3" s="174" t="s">
         <v>144</v>
       </c>
-      <c r="B3" s="167"/>
-      <c r="C3" s="167"/>
-      <c r="D3" s="167"/>
-      <c r="E3" s="167"/>
-      <c r="F3" s="167"/>
-      <c r="G3" s="167"/>
-      <c r="H3" s="167"/>
-      <c r="I3" s="167"/>
-      <c r="J3" s="167"/>
-      <c r="K3" s="167"/>
-      <c r="L3" s="167"/>
-      <c r="M3" s="167"/>
-      <c r="N3" s="167"/>
-      <c r="O3" s="167"/>
-      <c r="P3" s="167"/>
-      <c r="Q3" s="167"/>
+      <c r="B3" s="174"/>
+      <c r="C3" s="174"/>
+      <c r="D3" s="174"/>
+      <c r="E3" s="174"/>
+      <c r="F3" s="174"/>
+      <c r="G3" s="174"/>
+      <c r="H3" s="174"/>
+      <c r="I3" s="174"/>
+      <c r="J3" s="174"/>
+      <c r="K3" s="174"/>
+      <c r="L3" s="174"/>
+      <c r="M3" s="174"/>
+      <c r="N3" s="174"/>
+      <c r="O3" s="174"/>
+      <c r="P3" s="174"/>
+      <c r="Q3" s="174"/>
     </row>
     <row r="4" spans="1:17" ht="14.4">
-      <c r="A4" s="169" t="s">
+      <c r="A4" s="176" t="s">
         <v>145</v>
       </c>
-      <c r="B4" s="169"/>
-      <c r="C4" s="169"/>
+      <c r="B4" s="176"/>
+      <c r="C4" s="176"/>
       <c r="D4" s="69"/>
       <c r="E4" s="69"/>
       <c r="F4" s="69"/>
@@ -9651,11 +9651,11 @@
       <c r="Q4" s="70"/>
     </row>
     <row r="5" spans="1:17" ht="14.4">
-      <c r="A5" s="168" t="s">
+      <c r="A5" s="175" t="s">
         <v>146</v>
       </c>
-      <c r="B5" s="168"/>
-      <c r="C5" s="168"/>
+      <c r="B5" s="175"/>
+      <c r="C5" s="175"/>
       <c r="D5" s="69"/>
       <c r="E5" s="69"/>
       <c r="F5" s="69"/>
@@ -11195,20 +11195,20 @@
       <c r="G1" s="129" t="s">
         <v>306</v>
       </c>
-      <c r="J1" s="171" t="s">
+      <c r="J1" s="166" t="s">
         <v>307</v>
       </c>
-      <c r="K1" s="172"/>
-      <c r="L1" s="172"/>
-      <c r="M1" s="173"/>
-      <c r="P1" s="174" t="s">
+      <c r="K1" s="167"/>
+      <c r="L1" s="167"/>
+      <c r="M1" s="168"/>
+      <c r="P1" s="169" t="s">
         <v>308</v>
       </c>
-      <c r="Q1" s="175"/>
-      <c r="R1" s="175"/>
-      <c r="S1" s="175"/>
-      <c r="T1" s="175"/>
-      <c r="U1" s="176"/>
+      <c r="Q1" s="170"/>
+      <c r="R1" s="170"/>
+      <c r="S1" s="170"/>
+      <c r="T1" s="170"/>
+      <c r="U1" s="171"/>
     </row>
     <row r="2" spans="1:21">
       <c r="A2" s="105">
@@ -11224,11 +11224,11 @@
         <v>3</v>
       </c>
       <c r="D2" s="106">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E2" s="106" t="str">
         <f>IF(D2=0,"Open",IF(D2=C2,"Done","InProgress"))</f>
-        <v>Open</v>
+        <v>Done</v>
       </c>
       <c r="F2" s="106" t="str">
         <f>'UAT Scenarios'!H7</f>
@@ -11257,7 +11257,7 @@
       </c>
       <c r="R2" s="133"/>
       <c r="T2" s="153"/>
-      <c r="U2" s="170" t="s">
+      <c r="U2" s="165" t="s">
         <v>312</v>
       </c>
     </row>
@@ -11275,11 +11275,11 @@
         <v>3</v>
       </c>
       <c r="D3" s="106">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E3" s="106" t="str">
         <f t="shared" ref="E3:E26" si="0">IF(D3=0,"Open",IF(D3=C3,"Done","InProgress"))</f>
-        <v>Open</v>
+        <v>Done</v>
       </c>
       <c r="F3" s="106" t="str">
         <f>'UAT Scenarios'!H8</f>
@@ -11308,7 +11308,7 @@
         <v>315</v>
       </c>
       <c r="T3" s="153"/>
-      <c r="U3" s="170"/>
+      <c r="U3" s="165"/>
     </row>
     <row r="4" spans="1:21">
       <c r="A4" s="105">
@@ -11323,11 +11323,11 @@
         <v>3</v>
       </c>
       <c r="D4" s="106">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E4" s="106" t="str">
         <f t="shared" si="0"/>
-        <v>Open</v>
+        <v>Done</v>
       </c>
       <c r="F4" s="106" t="str">
         <f>'UAT Scenarios'!H9</f>
@@ -11375,11 +11375,11 @@
         <v>3</v>
       </c>
       <c r="D5" s="106">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E5" s="106" t="str">
         <f t="shared" si="0"/>
-        <v>Open</v>
+        <v>Done</v>
       </c>
       <c r="F5" s="106" t="str">
         <f>'UAT Scenarios'!H10</f>
@@ -11430,11 +11430,11 @@
         <v>2</v>
       </c>
       <c r="D6" s="106">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" s="106" t="str">
         <f t="shared" si="0"/>
-        <v>Open</v>
+        <v>Done</v>
       </c>
       <c r="F6" s="106" t="str">
         <f>'UAT Scenarios'!H11</f>

</xml_diff>